<commit_message>
Normalize aum diff values to numeric-only format.
Remove 'cr' suffix from aum diff while preserving sign and numeric denomination so peer table metrics use consistent numeric text.
</commit_message>
<xml_diff>
--- a/MF analysis structure test/data/matched_only_sorted.xlsx
+++ b/MF analysis structure test/data/matched_only_sorted.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4680" yWindow="660" windowWidth="24720" windowHeight="17260" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4680" yWindow="660" windowWidth="24720" windowHeight="17160" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="matched_only" sheetId="1" state="visible" r:id="rId1"/>
@@ -1034,7 +1034,7 @@
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>1cr</t>
+          <t>1</t>
         </is>
       </c>
       <c r="AY2" s="26" t="n">
@@ -1194,7 +1194,7 @@
       </c>
       <c r="AX3" s="18" t="inlineStr">
         <is>
-          <t>-46cr</t>
+          <t>-46</t>
         </is>
       </c>
       <c r="AY3" s="26" t="n">
@@ -1390,7 +1390,7 @@
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>16cr</t>
+          <t>16</t>
         </is>
       </c>
       <c r="AY4" s="26" t="n">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="AX5" s="18" t="inlineStr">
         <is>
-          <t>-127cr</t>
+          <t>-127</t>
         </is>
       </c>
       <c r="AY5" s="26" t="n">
@@ -1770,7 +1770,7 @@
       </c>
       <c r="AX6" t="inlineStr">
         <is>
-          <t>62cr</t>
+          <t>62</t>
         </is>
       </c>
       <c r="AY6" s="26" t="n">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="AX7" s="18" t="inlineStr">
         <is>
-          <t>-13cr</t>
+          <t>-13</t>
         </is>
       </c>
       <c r="AY7" s="26" t="n">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="AX8" s="18" t="inlineStr">
         <is>
-          <t>-94cr</t>
+          <t>-94</t>
         </is>
       </c>
       <c r="AY8" s="26" t="n">
@@ -2286,7 +2286,7 @@
       </c>
       <c r="AX9" s="18" t="inlineStr">
         <is>
-          <t>-2cr</t>
+          <t>-2</t>
         </is>
       </c>
       <c r="AY9" s="26" t="n">
@@ -2571,7 +2571,7 @@
       </c>
       <c r="AX11" s="18" t="inlineStr">
         <is>
-          <t>-238cr</t>
+          <t>-238</t>
         </is>
       </c>
       <c r="AY11" s="26" t="n">
@@ -2767,7 +2767,7 @@
       </c>
       <c r="AX12" s="18" t="inlineStr">
         <is>
-          <t>-835cr</t>
+          <t>-835</t>
         </is>
       </c>
       <c r="AY12" s="26" t="n">
@@ -2907,7 +2907,7 @@
       </c>
       <c r="AX13" t="inlineStr">
         <is>
-          <t>1cr</t>
+          <t>1</t>
         </is>
       </c>
       <c r="AY13" s="26" t="n">
@@ -3103,7 +3103,7 @@
       </c>
       <c r="AX14" t="inlineStr">
         <is>
-          <t>4cr</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AY14" s="26" t="n">
@@ -3299,7 +3299,7 @@
       </c>
       <c r="AX15" s="18" t="inlineStr">
         <is>
-          <t>-9cr</t>
+          <t>-9</t>
         </is>
       </c>
       <c r="AY15" s="26" t="n">
@@ -3495,7 +3495,7 @@
       </c>
       <c r="AX16" s="18" t="inlineStr">
         <is>
-          <t>-9cr</t>
+          <t>-9</t>
         </is>
       </c>
       <c r="AY16" s="26" t="n">
@@ -3691,7 +3691,7 @@
       </c>
       <c r="AX17" t="inlineStr">
         <is>
-          <t>3cr</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AY17" s="26" t="n">
@@ -3887,7 +3887,7 @@
       </c>
       <c r="AX18" s="18" t="inlineStr">
         <is>
-          <t>-73cr</t>
+          <t>-73</t>
         </is>
       </c>
       <c r="AY18" s="26" t="n">
@@ -4071,7 +4071,7 @@
       </c>
       <c r="AX19" t="inlineStr">
         <is>
-          <t>0cr</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY19" s="26" t="n">
@@ -4265,7 +4265,7 @@
       </c>
       <c r="AX20" s="18" t="inlineStr">
         <is>
-          <t>-85cr</t>
+          <t>-85</t>
         </is>
       </c>
       <c r="AY20" s="26" t="n">
@@ -4461,7 +4461,7 @@
       </c>
       <c r="AX21" s="18" t="inlineStr">
         <is>
-          <t>-52cr</t>
+          <t>-52</t>
         </is>
       </c>
       <c r="AY21" s="26" t="n">
@@ -4657,7 +4657,7 @@
       </c>
       <c r="AX22" s="18" t="inlineStr">
         <is>
-          <t>-168cr</t>
+          <t>-168</t>
         </is>
       </c>
       <c r="AY22" s="26" t="n">
@@ -4853,7 +4853,7 @@
       </c>
       <c r="AX23" s="18" t="inlineStr">
         <is>
-          <t>-55cr</t>
+          <t>-55</t>
         </is>
       </c>
       <c r="AY23" s="26" t="n">
@@ -5037,7 +5037,7 @@
       </c>
       <c r="AX24" t="inlineStr">
         <is>
-          <t>2cr</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AY24" s="26" t="n">
@@ -5233,7 +5233,7 @@
       </c>
       <c r="AX25" s="18" t="inlineStr">
         <is>
-          <t>-2cr</t>
+          <t>-2</t>
         </is>
       </c>
       <c r="AY25" s="26" t="n">
@@ -5429,7 +5429,7 @@
       </c>
       <c r="AX26" s="18" t="inlineStr">
         <is>
-          <t>-36cr</t>
+          <t>-36</t>
         </is>
       </c>
       <c r="AY26" s="26" t="n">
@@ -5625,7 +5625,7 @@
       </c>
       <c r="AX27" s="18" t="inlineStr">
         <is>
-          <t>-4cr</t>
+          <t>-4</t>
         </is>
       </c>
       <c r="AY27" s="26" t="n">
@@ -5809,7 +5809,7 @@
       </c>
       <c r="AX28" s="18" t="inlineStr">
         <is>
-          <t>-4cr</t>
+          <t>-4</t>
         </is>
       </c>
       <c r="AY28" s="26" t="n">
@@ -6005,7 +6005,7 @@
       </c>
       <c r="AX29" s="18" t="inlineStr">
         <is>
-          <t>-40cr</t>
+          <t>-40</t>
         </is>
       </c>
       <c r="AY29" s="26" t="n">
@@ -6201,7 +6201,7 @@
       </c>
       <c r="AX30" s="18" t="inlineStr">
         <is>
-          <t>-114cr</t>
+          <t>-114</t>
         </is>
       </c>
       <c r="AY30" s="26" t="n">
@@ -6397,7 +6397,7 @@
       </c>
       <c r="AX31" s="18" t="inlineStr">
         <is>
-          <t>-1cr</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="AY31" s="26" t="n">
@@ -6593,7 +6593,7 @@
       </c>
       <c r="AX32" s="18" t="inlineStr">
         <is>
-          <t>-230cr</t>
+          <t>-230</t>
         </is>
       </c>
       <c r="AY32" s="26" t="n">
@@ -6753,7 +6753,7 @@
       </c>
       <c r="AX33" t="inlineStr">
         <is>
-          <t>2cr</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AY33" s="26" t="n">
@@ -6937,7 +6937,7 @@
       </c>
       <c r="AX34" t="inlineStr">
         <is>
-          <t>40cr</t>
+          <t>40</t>
         </is>
       </c>
       <c r="AY34" s="26" t="n">
@@ -7133,7 +7133,7 @@
       </c>
       <c r="AX35" s="18" t="inlineStr">
         <is>
-          <t>-15cr</t>
+          <t>-15</t>
         </is>
       </c>
       <c r="AY35" s="26" t="n">
@@ -7329,7 +7329,7 @@
       </c>
       <c r="AX36" s="18" t="inlineStr">
         <is>
-          <t>-115cr</t>
+          <t>-115</t>
         </is>
       </c>
       <c r="AY36" s="26" t="n">
@@ -7521,7 +7521,7 @@
       </c>
       <c r="AX37" t="inlineStr">
         <is>
-          <t>2cr</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AY37" s="26" t="n">
@@ -7715,7 +7715,7 @@
       </c>
       <c r="AX38" t="inlineStr">
         <is>
-          <t>326cr</t>
+          <t>326</t>
         </is>
       </c>
       <c r="AY38" s="26" t="n">
@@ -7899,7 +7899,7 @@
       </c>
       <c r="AX39" t="inlineStr">
         <is>
-          <t>0cr</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY39" s="26" t="n">
@@ -8093,7 +8093,7 @@
       </c>
       <c r="AX40" s="18" t="inlineStr">
         <is>
-          <t>-5cr</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="AY40" s="26" t="n">
@@ -8287,7 +8287,7 @@
       </c>
       <c r="AX41" s="18" t="inlineStr">
         <is>
-          <t>-2cr</t>
+          <t>-2</t>
         </is>
       </c>
       <c r="AY41" s="26" t="n">
@@ -8459,7 +8459,7 @@
       </c>
       <c r="AX42" s="18" t="inlineStr">
         <is>
-          <t>-2cr</t>
+          <t>-2</t>
         </is>
       </c>
       <c r="AY42" s="26" t="n">
@@ -8739,7 +8739,7 @@
       </c>
       <c r="AX44" t="inlineStr">
         <is>
-          <t>288cr</t>
+          <t>288</t>
         </is>
       </c>
       <c r="AY44" s="26" t="n">
@@ -8923,7 +8923,7 @@
       </c>
       <c r="AX45" s="18" t="inlineStr">
         <is>
-          <t>-255cr</t>
+          <t>-255</t>
         </is>
       </c>
       <c r="AY45" s="26" t="n">
@@ -9083,7 +9083,7 @@
       </c>
       <c r="AX46" t="inlineStr">
         <is>
-          <t>92cr</t>
+          <t>92</t>
         </is>
       </c>
       <c r="AY46" s="26" t="n">
@@ -9277,7 +9277,7 @@
       </c>
       <c r="AX47" s="18" t="inlineStr">
         <is>
-          <t>-29cr</t>
+          <t>-29</t>
         </is>
       </c>
       <c r="AY47" s="26" t="n">
@@ -9461,7 +9461,7 @@
       </c>
       <c r="AX48" s="18" t="inlineStr">
         <is>
-          <t>-9cr</t>
+          <t>-9</t>
         </is>
       </c>
       <c r="AY48" s="26" t="n">
@@ -9633,7 +9633,7 @@
       </c>
       <c r="AX49" s="18" t="inlineStr">
         <is>
-          <t>-18cr</t>
+          <t>-18</t>
         </is>
       </c>
       <c r="AY49" s="26" t="n">
@@ -9827,7 +9827,7 @@
       </c>
       <c r="AX50" s="18" t="inlineStr">
         <is>
-          <t>-139cr</t>
+          <t>-139</t>
         </is>
       </c>
       <c r="AY50" s="26" t="n">
@@ -10023,7 +10023,7 @@
       </c>
       <c r="AX51" t="inlineStr">
         <is>
-          <t>62cr</t>
+          <t>62</t>
         </is>
       </c>
       <c r="AY51" s="26" t="n">
@@ -10217,7 +10217,7 @@
       </c>
       <c r="AX52" t="inlineStr">
         <is>
-          <t>6cr</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AY52" s="26" t="n">
@@ -10411,7 +10411,7 @@
       </c>
       <c r="AX53" t="inlineStr">
         <is>
-          <t>2402cr</t>
+          <t>2402</t>
         </is>
       </c>
       <c r="AY53" s="26" t="n">
@@ -10571,7 +10571,7 @@
       </c>
       <c r="AX54" t="inlineStr">
         <is>
-          <t>438cr</t>
+          <t>438</t>
         </is>
       </c>
       <c r="AY54" s="26" t="n">
@@ -10767,7 +10767,7 @@
       </c>
       <c r="AX55" s="18" t="inlineStr">
         <is>
-          <t>-16cr</t>
+          <t>-16</t>
         </is>
       </c>
       <c r="AY55" s="26" t="n">
@@ -10939,7 +10939,7 @@
       </c>
       <c r="AX56" t="inlineStr">
         <is>
-          <t>75cr</t>
+          <t>75</t>
         </is>
       </c>
       <c r="AY56" s="26" t="n">
@@ -11111,7 +11111,7 @@
       </c>
       <c r="AX57" t="inlineStr">
         <is>
-          <t>68cr</t>
+          <t>68</t>
         </is>
       </c>
       <c r="AY57" s="26" t="n">
@@ -11271,7 +11271,7 @@
       </c>
       <c r="AX58" t="inlineStr">
         <is>
-          <t>0cr</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY58" s="26" t="n">
@@ -11409,7 +11409,7 @@
       </c>
       <c r="AX59" t="inlineStr">
         <is>
-          <t>272cr</t>
+          <t>272</t>
         </is>
       </c>
       <c r="AY59" s="26" t="n">
@@ -11581,7 +11581,7 @@
       </c>
       <c r="AX60" t="inlineStr">
         <is>
-          <t>0cr</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY60" s="26" t="n">
@@ -11741,7 +11741,7 @@
       </c>
       <c r="AX61" t="inlineStr">
         <is>
-          <t>107cr</t>
+          <t>107</t>
         </is>
       </c>
       <c r="AY61" s="26" t="n">
@@ -11937,7 +11937,7 @@
       </c>
       <c r="AX62" s="18" t="inlineStr">
         <is>
-          <t>-433cr</t>
+          <t>-433</t>
         </is>
       </c>
       <c r="AY62" s="26" t="n">
@@ -12121,7 +12121,7 @@
       </c>
       <c r="AX63" s="18" t="inlineStr">
         <is>
-          <t>-1cr</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="AY63" s="26" t="n">
@@ -12293,7 +12293,7 @@
       </c>
       <c r="AX64" s="18" t="inlineStr">
         <is>
-          <t>-13cr</t>
+          <t>-13</t>
         </is>
       </c>
       <c r="AY64" s="26" t="n">
@@ -12453,7 +12453,7 @@
       </c>
       <c r="AX65" t="inlineStr">
         <is>
-          <t>21cr</t>
+          <t>21</t>
         </is>
       </c>
       <c r="AY65" s="26" t="n">
@@ -12649,7 +12649,7 @@
       </c>
       <c r="AX66" t="inlineStr">
         <is>
-          <t>3232cr</t>
+          <t>3232</t>
         </is>
       </c>
       <c r="AY66" s="26" t="n">
@@ -12833,7 +12833,7 @@
       </c>
       <c r="AX67" s="18" t="inlineStr">
         <is>
-          <t>-1cr</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="AY67" s="26" t="n">
@@ -13017,7 +13017,7 @@
       </c>
       <c r="AX68" t="inlineStr">
         <is>
-          <t>39cr</t>
+          <t>39</t>
         </is>
       </c>
       <c r="AY68" s="26" t="n">
@@ -13211,7 +13211,7 @@
       </c>
       <c r="AX69" s="18" t="inlineStr">
         <is>
-          <t>-8cr</t>
+          <t>-8</t>
         </is>
       </c>
       <c r="AY69" s="26" t="n">
@@ -13371,7 +13371,7 @@
       </c>
       <c r="AX70" s="18" t="inlineStr">
         <is>
-          <t>-19cr</t>
+          <t>-19</t>
         </is>
       </c>
       <c r="AY70" s="26" t="n">
@@ -13701,7 +13701,7 @@
       </c>
       <c r="AX72" s="18" t="inlineStr">
         <is>
-          <t>-12cr</t>
+          <t>-12</t>
         </is>
       </c>
       <c r="AY72" s="26" t="n">
@@ -13873,7 +13873,7 @@
       </c>
       <c r="AX73" t="inlineStr">
         <is>
-          <t>247cr</t>
+          <t>247</t>
         </is>
       </c>
       <c r="AY73" s="26" t="n">
@@ -14153,7 +14153,7 @@
       </c>
       <c r="AX75" s="18" t="inlineStr">
         <is>
-          <t>-18cr</t>
+          <t>-18</t>
         </is>
       </c>
       <c r="AY75" s="26" t="n">
@@ -14337,7 +14337,7 @@
       </c>
       <c r="AX76" t="inlineStr">
         <is>
-          <t>6cr</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AY76" s="26" t="n">
@@ -14497,7 +14497,7 @@
       </c>
       <c r="AX77" t="inlineStr">
         <is>
-          <t>46cr</t>
+          <t>46</t>
         </is>
       </c>
       <c r="AY77" s="26" t="n">
@@ -14693,7 +14693,7 @@
       </c>
       <c r="AX78" t="inlineStr">
         <is>
-          <t>891cr</t>
+          <t>891</t>
         </is>
       </c>
       <c r="AY78" s="26" t="n">
@@ -14889,7 +14889,7 @@
       </c>
       <c r="AX79" t="inlineStr">
         <is>
-          <t>8cr</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AY79" s="26" t="n">
@@ -15083,7 +15083,7 @@
       </c>
       <c r="AX80" s="18" t="inlineStr">
         <is>
-          <t>-558cr</t>
+          <t>-558</t>
         </is>
       </c>
       <c r="AY80" s="26" t="n">
@@ -15277,7 +15277,7 @@
       </c>
       <c r="AX81" s="18" t="inlineStr">
         <is>
-          <t>-24cr</t>
+          <t>-24</t>
         </is>
       </c>
       <c r="AY81" s="26" t="n">
@@ -15471,7 +15471,7 @@
       </c>
       <c r="AX82" t="inlineStr">
         <is>
-          <t>221cr</t>
+          <t>221</t>
         </is>
       </c>
       <c r="AY82" s="26" t="n">
@@ -15631,7 +15631,7 @@
       </c>
       <c r="AX83" t="inlineStr">
         <is>
-          <t>47cr</t>
+          <t>47</t>
         </is>
       </c>
       <c r="AY83" s="26" t="n">
@@ -15825,7 +15825,7 @@
       </c>
       <c r="AX84" t="inlineStr">
         <is>
-          <t>921cr</t>
+          <t>921</t>
         </is>
       </c>
       <c r="AY84" s="26" t="n">
@@ -16021,7 +16021,7 @@
       </c>
       <c r="AX85" t="inlineStr">
         <is>
-          <t>32cr</t>
+          <t>32</t>
         </is>
       </c>
       <c r="AY85" s="26" t="n">
@@ -16181,7 +16181,7 @@
       </c>
       <c r="AX86" s="18" t="inlineStr">
         <is>
-          <t>-35cr</t>
+          <t>-35</t>
         </is>
       </c>
       <c r="AY86" s="26" t="n">
@@ -16321,7 +16321,7 @@
       </c>
       <c r="AX87" t="inlineStr">
         <is>
-          <t>10cr</t>
+          <t>10</t>
         </is>
       </c>
       <c r="AY87" s="26" t="n">
@@ -16515,7 +16515,7 @@
       </c>
       <c r="AX88" t="inlineStr">
         <is>
-          <t>204cr</t>
+          <t>204</t>
         </is>
       </c>
       <c r="AY88" s="26" t="n">
@@ -16711,7 +16711,7 @@
       </c>
       <c r="AX89" s="18" t="inlineStr">
         <is>
-          <t>-16cr</t>
+          <t>-16</t>
         </is>
       </c>
       <c r="AY89" s="26" t="n">
@@ -16895,7 +16895,7 @@
       </c>
       <c r="AX90" t="inlineStr">
         <is>
-          <t>3cr</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AY90" s="26" t="n">
@@ -17091,7 +17091,7 @@
       </c>
       <c r="AX91" t="inlineStr">
         <is>
-          <t>289cr</t>
+          <t>289</t>
         </is>
       </c>
       <c r="AY91" s="26" t="n">
@@ -17275,7 +17275,7 @@
       </c>
       <c r="AX92" s="18" t="inlineStr">
         <is>
-          <t>-90cr</t>
+          <t>-90</t>
         </is>
       </c>
       <c r="AY92" s="26" t="n">
@@ -17471,7 +17471,7 @@
       </c>
       <c r="AX93" s="18" t="inlineStr">
         <is>
-          <t>-3cr</t>
+          <t>-3</t>
         </is>
       </c>
       <c r="AY93" s="26" t="n">
@@ -17665,7 +17665,7 @@
       </c>
       <c r="AX94" t="inlineStr">
         <is>
-          <t>63cr</t>
+          <t>63</t>
         </is>
       </c>
       <c r="AY94" s="26" t="n">
@@ -17825,7 +17825,7 @@
       </c>
       <c r="AX95" s="18" t="inlineStr">
         <is>
-          <t>-2cr</t>
+          <t>-2</t>
         </is>
       </c>
       <c r="AY95" s="26" t="n">
@@ -18019,7 +18019,7 @@
       </c>
       <c r="AX96" s="18" t="inlineStr">
         <is>
-          <t>-75cr</t>
+          <t>-75</t>
         </is>
       </c>
       <c r="AY96" s="26" t="n">
@@ -18179,7 +18179,7 @@
       </c>
       <c r="AX97" t="inlineStr">
         <is>
-          <t>34cr</t>
+          <t>34</t>
         </is>
       </c>
       <c r="AY97" s="26" t="n">
@@ -18459,7 +18459,7 @@
       </c>
       <c r="AX99" t="inlineStr">
         <is>
-          <t>72cr</t>
+          <t>72</t>
         </is>
       </c>
       <c r="AY99" s="26" t="n">
@@ -18655,7 +18655,7 @@
       </c>
       <c r="AX100" s="18" t="inlineStr">
         <is>
-          <t>-531cr</t>
+          <t>-531</t>
         </is>
       </c>
       <c r="AY100" s="26" t="n">
@@ -18815,7 +18815,7 @@
       </c>
       <c r="AX101" s="18" t="inlineStr">
         <is>
-          <t>-96cr</t>
+          <t>-96</t>
         </is>
       </c>
       <c r="AY101" s="26" t="n">
@@ -19009,7 +19009,7 @@
       </c>
       <c r="AX102" t="inlineStr">
         <is>
-          <t>6cr</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AY102" s="26" t="n">
@@ -19181,7 +19181,7 @@
       </c>
       <c r="AX103" t="inlineStr">
         <is>
-          <t>1cr</t>
+          <t>1</t>
         </is>
       </c>
       <c r="AY103" s="26" t="n">
@@ -19377,7 +19377,7 @@
       </c>
       <c r="AX104" s="18" t="inlineStr">
         <is>
-          <t>-81cr</t>
+          <t>-81</t>
         </is>
       </c>
       <c r="AY104" s="26" t="n">
@@ -19573,7 +19573,7 @@
       </c>
       <c r="AX105" s="18" t="inlineStr">
         <is>
-          <t>-12cr</t>
+          <t>-12</t>
         </is>
       </c>
       <c r="AY105" s="26" t="n">
@@ -19769,7 +19769,7 @@
       </c>
       <c r="AX106" t="inlineStr">
         <is>
-          <t>14cr</t>
+          <t>14</t>
         </is>
       </c>
       <c r="AY106" s="26" t="n">
@@ -19963,7 +19963,7 @@
       </c>
       <c r="AX107" s="18" t="inlineStr">
         <is>
-          <t>-52cr</t>
+          <t>-52</t>
         </is>
       </c>
       <c r="AY107" s="26" t="n">
@@ -20159,7 +20159,7 @@
       </c>
       <c r="AX108" t="inlineStr">
         <is>
-          <t>0cr</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY108" s="26" t="n">
@@ -20353,7 +20353,7 @@
       </c>
       <c r="AX109" t="inlineStr">
         <is>
-          <t>149cr</t>
+          <t>149</t>
         </is>
       </c>
       <c r="AY109" s="26" t="n">
@@ -20547,7 +20547,7 @@
       </c>
       <c r="AX110" t="inlineStr">
         <is>
-          <t>2cr</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AY110" s="26" t="n">
@@ -20743,7 +20743,7 @@
       </c>
       <c r="AX111" t="inlineStr">
         <is>
-          <t>1cr</t>
+          <t>1</t>
         </is>
       </c>
       <c r="AY111" s="26" t="n">
@@ -20927,7 +20927,7 @@
       </c>
       <c r="AX112" s="18" t="inlineStr">
         <is>
-          <t>-2cr</t>
+          <t>-2</t>
         </is>
       </c>
       <c r="AY112" s="26" t="n">
@@ -21121,7 +21121,7 @@
       </c>
       <c r="AX113" s="18" t="inlineStr">
         <is>
-          <t>-18cr</t>
+          <t>-18</t>
         </is>
       </c>
       <c r="AY113" s="26" t="n">
@@ -21315,7 +21315,7 @@
       </c>
       <c r="AX114" t="inlineStr">
         <is>
-          <t>23cr</t>
+          <t>23</t>
         </is>
       </c>
       <c r="AY114" s="26" t="n">
@@ -21509,7 +21509,7 @@
       </c>
       <c r="AX115" s="18" t="inlineStr">
         <is>
-          <t>-7cr</t>
+          <t>-7</t>
         </is>
       </c>
       <c r="AY115" s="26" t="n">
@@ -21693,7 +21693,7 @@
       </c>
       <c r="AX116" t="inlineStr">
         <is>
-          <t>10cr</t>
+          <t>10</t>
         </is>
       </c>
       <c r="AY116" s="26" t="n">
@@ -21889,7 +21889,7 @@
       </c>
       <c r="AX117" s="18" t="inlineStr">
         <is>
-          <t>-28cr</t>
+          <t>-28</t>
         </is>
       </c>
       <c r="AY117" s="26" t="n">
@@ -22049,7 +22049,7 @@
       </c>
       <c r="AX118" t="inlineStr">
         <is>
-          <t>54cr</t>
+          <t>54</t>
         </is>
       </c>
       <c r="AZ118" s="26" t="n">
@@ -22239,7 +22239,7 @@
       </c>
       <c r="AX119" t="inlineStr">
         <is>
-          <t>678cr</t>
+          <t>678</t>
         </is>
       </c>
       <c r="AY119" s="26" t="n">
@@ -22435,7 +22435,7 @@
       </c>
       <c r="AX120" s="18" t="inlineStr">
         <is>
-          <t>-7cr</t>
+          <t>-7</t>
         </is>
       </c>
       <c r="AY120" s="26" t="n">
@@ -22629,7 +22629,7 @@
       </c>
       <c r="AX121" t="inlineStr">
         <is>
-          <t>418cr</t>
+          <t>418</t>
         </is>
       </c>
       <c r="AY121" s="26" t="n">
@@ -22823,7 +22823,7 @@
       </c>
       <c r="AX122" t="inlineStr">
         <is>
-          <t>23cr</t>
+          <t>23</t>
         </is>
       </c>
       <c r="AY122" s="26" t="n">
@@ -23017,7 +23017,7 @@
       </c>
       <c r="AX123" t="inlineStr">
         <is>
-          <t>0cr</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY123" s="26" t="n">
@@ -23201,7 +23201,7 @@
       </c>
       <c r="AX124" s="18" t="inlineStr">
         <is>
-          <t>-7cr</t>
+          <t>-7</t>
         </is>
       </c>
       <c r="AY124" s="26" t="n">
@@ -23373,7 +23373,7 @@
       </c>
       <c r="AX125" s="15" t="inlineStr">
         <is>
-          <t>6cr</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AY125" s="26" t="n">
@@ -23635,7 +23635,7 @@
       </c>
       <c r="AX127" s="18" t="inlineStr">
         <is>
-          <t>-491cr</t>
+          <t>-491</t>
         </is>
       </c>
       <c r="AY127" s="26" t="n">
@@ -23775,7 +23775,7 @@
       </c>
       <c r="AX128" s="18" t="inlineStr">
         <is>
-          <t>-8cr</t>
+          <t>-8</t>
         </is>
       </c>
       <c r="AY128" s="26" t="n">
@@ -23971,7 +23971,7 @@
       </c>
       <c r="AX129" s="18" t="inlineStr">
         <is>
-          <t>-8cr</t>
+          <t>-8</t>
         </is>
       </c>
       <c r="AY129" s="26" t="n">
@@ -24131,7 +24131,7 @@
       </c>
       <c r="AX130" t="inlineStr">
         <is>
-          <t>80cr</t>
+          <t>80</t>
         </is>
       </c>
       <c r="AY130" s="26" t="n">
@@ -24327,7 +24327,7 @@
       </c>
       <c r="AX131" t="inlineStr">
         <is>
-          <t>461cr</t>
+          <t>461</t>
         </is>
       </c>
       <c r="AY131" s="26" t="n">
@@ -24521,7 +24521,7 @@
       </c>
       <c r="AX132" s="18" t="inlineStr">
         <is>
-          <t>-53cr</t>
+          <t>-53</t>
         </is>
       </c>
       <c r="AY132" s="26" t="n">
@@ -24717,7 +24717,7 @@
       </c>
       <c r="AX133" t="inlineStr">
         <is>
-          <t>696cr</t>
+          <t>696</t>
         </is>
       </c>
       <c r="AY133" s="26" t="n">
@@ -24857,7 +24857,7 @@
       </c>
       <c r="AX134" t="inlineStr">
         <is>
-          <t>543cr</t>
+          <t>543</t>
         </is>
       </c>
       <c r="AY134" s="26" t="n">
@@ -25051,7 +25051,7 @@
       </c>
       <c r="AX135" t="inlineStr">
         <is>
-          <t>108cr</t>
+          <t>108</t>
         </is>
       </c>
       <c r="AY135" s="26" t="n">
@@ -25223,7 +25223,7 @@
       </c>
       <c r="AX136" t="inlineStr">
         <is>
-          <t>19cr</t>
+          <t>19</t>
         </is>
       </c>
       <c r="AY136" s="26" t="n">
@@ -25395,7 +25395,7 @@
       </c>
       <c r="AX137" s="18" t="inlineStr">
         <is>
-          <t>-297cr</t>
+          <t>-297</t>
         </is>
       </c>
       <c r="AY137" s="26" t="n">
@@ -25591,7 +25591,7 @@
       </c>
       <c r="AX138" t="inlineStr">
         <is>
-          <t>427cr</t>
+          <t>427</t>
         </is>
       </c>
       <c r="AY138" s="26" t="n">
@@ -25775,7 +25775,7 @@
       </c>
       <c r="AX139" t="inlineStr">
         <is>
-          <t>61cr</t>
+          <t>61</t>
         </is>
       </c>
       <c r="AY139" s="26" t="n">
@@ -25959,7 +25959,7 @@
       </c>
       <c r="AX140" t="inlineStr">
         <is>
-          <t>109cr</t>
+          <t>109</t>
         </is>
       </c>
       <c r="AY140" s="26" t="n">
@@ -26155,7 +26155,7 @@
       </c>
       <c r="AX141" s="18" t="inlineStr">
         <is>
-          <t>-1075cr</t>
+          <t>-1075</t>
         </is>
       </c>
       <c r="AY141" s="26" t="n">
@@ -26349,7 +26349,7 @@
       </c>
       <c r="AX142" t="inlineStr">
         <is>
-          <t>336cr</t>
+          <t>336</t>
         </is>
       </c>
       <c r="AY142" s="26" t="n">
@@ -26545,7 +26545,7 @@
       </c>
       <c r="AX143" s="18" t="inlineStr">
         <is>
-          <t>-250cr</t>
+          <t>-250</t>
         </is>
       </c>
       <c r="AY143" s="26" t="n">
@@ -26739,7 +26739,7 @@
       </c>
       <c r="AX144" t="inlineStr">
         <is>
-          <t>82cr</t>
+          <t>82</t>
         </is>
       </c>
       <c r="AY144" s="26" t="n">
@@ -26933,7 +26933,7 @@
       </c>
       <c r="AX145" s="18" t="inlineStr">
         <is>
-          <t>-38cr</t>
+          <t>-38</t>
         </is>
       </c>
       <c r="AY145" s="26" t="n">
@@ -27127,7 +27127,7 @@
       </c>
       <c r="AX146" t="inlineStr">
         <is>
-          <t>85cr</t>
+          <t>85</t>
         </is>
       </c>
       <c r="AY146" s="26" t="n">
@@ -27321,7 +27321,7 @@
       </c>
       <c r="AX147" s="18" t="inlineStr">
         <is>
-          <t>-2cr</t>
+          <t>-2</t>
         </is>
       </c>
       <c r="AY147" s="26" t="n">
@@ -27489,7 +27489,7 @@
       </c>
       <c r="AX148" t="inlineStr">
         <is>
-          <t>1cr</t>
+          <t>1</t>
         </is>
       </c>
       <c r="AY148" s="26" t="n">
@@ -27649,7 +27649,7 @@
       </c>
       <c r="AX149" t="inlineStr">
         <is>
-          <t>105cr</t>
+          <t>105</t>
         </is>
       </c>
       <c r="AY149" s="26" t="n">
@@ -27907,7 +27907,7 @@
       </c>
       <c r="AX151" t="inlineStr">
         <is>
-          <t>33cr</t>
+          <t>33</t>
         </is>
       </c>
       <c r="AY151" s="26" t="n">
@@ -28047,7 +28047,7 @@
       </c>
       <c r="AX152" t="inlineStr">
         <is>
-          <t>45cr</t>
+          <t>45</t>
         </is>
       </c>
       <c r="AY152" s="26" t="n">
@@ -28241,7 +28241,7 @@
       </c>
       <c r="AX153" t="inlineStr">
         <is>
-          <t>2cr</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AY153" s="26" t="n">
@@ -28401,7 +28401,7 @@
       </c>
       <c r="AX154" t="inlineStr">
         <is>
-          <t>119cr</t>
+          <t>119</t>
         </is>
       </c>
       <c r="AY154" s="26" t="n">
@@ -28561,7 +28561,7 @@
       </c>
       <c r="AX155" t="inlineStr">
         <is>
-          <t>27cr</t>
+          <t>27</t>
         </is>
       </c>
       <c r="AY155" s="26" t="n">
@@ -28721,7 +28721,7 @@
       </c>
       <c r="AX156" s="18" t="inlineStr">
         <is>
-          <t>-89cr</t>
+          <t>-89</t>
         </is>
       </c>
       <c r="AY156" s="26" t="n">
@@ -28881,7 +28881,7 @@
       </c>
       <c r="AX157" t="inlineStr">
         <is>
-          <t>30cr</t>
+          <t>30</t>
         </is>
       </c>
       <c r="AY157" s="26" t="n">
@@ -29041,7 +29041,7 @@
       </c>
       <c r="AX158" s="18" t="inlineStr">
         <is>
-          <t>-28cr</t>
+          <t>-28</t>
         </is>
       </c>
       <c r="AY158" s="26" t="n">
@@ -29235,7 +29235,7 @@
       </c>
       <c r="AX159" t="inlineStr">
         <is>
-          <t>203cr</t>
+          <t>203</t>
         </is>
       </c>
       <c r="AY159" s="26" t="n">
@@ -29431,7 +29431,7 @@
       </c>
       <c r="AX160" s="18" t="inlineStr">
         <is>
-          <t>-110cr</t>
+          <t>-110</t>
         </is>
       </c>
       <c r="AY160" s="26" t="n">
@@ -29615,7 +29615,7 @@
       </c>
       <c r="AX161" s="18" t="inlineStr">
         <is>
-          <t>-4cr</t>
+          <t>-4</t>
         </is>
       </c>
       <c r="AY161" s="26" t="n">
@@ -29787,7 +29787,7 @@
       </c>
       <c r="AX162" t="inlineStr">
         <is>
-          <t>827cr</t>
+          <t>827</t>
         </is>
       </c>
       <c r="AY162" s="26" t="n">
@@ -29959,7 +29959,7 @@
       </c>
       <c r="AX163" t="inlineStr">
         <is>
-          <t>8cr</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AY163" s="26" t="n">
@@ -30143,7 +30143,7 @@
       </c>
       <c r="AX164" t="inlineStr">
         <is>
-          <t>46cr</t>
+          <t>46</t>
         </is>
       </c>
       <c r="AY164" s="26" t="n">
@@ -30303,7 +30303,7 @@
       </c>
       <c r="AX165" t="inlineStr">
         <is>
-          <t>101cr</t>
+          <t>101</t>
         </is>
       </c>
       <c r="AY165" s="26" t="n">
@@ -30463,7 +30463,7 @@
       </c>
       <c r="AX166" s="18" t="inlineStr">
         <is>
-          <t>-211cr</t>
+          <t>-211</t>
         </is>
       </c>
       <c r="AY166" s="26" t="n">
@@ -30623,7 +30623,7 @@
       </c>
       <c r="AX167" s="18" t="inlineStr">
         <is>
-          <t>-9cr</t>
+          <t>-9</t>
         </is>
       </c>
       <c r="AY167" s="26" t="n">
@@ -30817,7 +30817,7 @@
       </c>
       <c r="AX168" s="18" t="inlineStr">
         <is>
-          <t>-616cr</t>
+          <t>-616</t>
         </is>
       </c>
       <c r="AY168" s="26" t="n">
@@ -30977,7 +30977,7 @@
       </c>
       <c r="AX169" t="inlineStr">
         <is>
-          <t>2cr</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AY169" s="26" t="n">
@@ -31149,7 +31149,7 @@
       </c>
       <c r="AX170" s="18" t="inlineStr">
         <is>
-          <t>-12cr</t>
+          <t>-12</t>
         </is>
       </c>
       <c r="AY170" s="26" t="n">
@@ -31309,7 +31309,7 @@
       </c>
       <c r="AX171" t="inlineStr">
         <is>
-          <t>118cr</t>
+          <t>118</t>
         </is>
       </c>
       <c r="AY171" s="26" t="n">
@@ -31567,7 +31567,7 @@
       </c>
       <c r="AX173" s="18" t="inlineStr">
         <is>
-          <t>-9cr</t>
+          <t>-9</t>
         </is>
       </c>
       <c r="AY173" s="26" t="n">
@@ -31913,7 +31913,7 @@
       </c>
       <c r="AX175" s="18" t="inlineStr">
         <is>
-          <t>-22cr</t>
+          <t>-22</t>
         </is>
       </c>
       <c r="AY175" s="26" t="n">
@@ -32107,7 +32107,7 @@
       </c>
       <c r="AX176" s="18" t="inlineStr">
         <is>
-          <t>-7cr</t>
+          <t>-7</t>
         </is>
       </c>
       <c r="AY176" s="26" t="n">
@@ -32291,7 +32291,7 @@
       </c>
       <c r="AX177" s="18" t="inlineStr">
         <is>
-          <t>-4cr</t>
+          <t>-4</t>
         </is>
       </c>
       <c r="AY177" s="26" t="n">
@@ -32487,7 +32487,7 @@
       </c>
       <c r="AX178" s="18" t="inlineStr">
         <is>
-          <t>-24cr</t>
+          <t>-24</t>
         </is>
       </c>
       <c r="AY178" s="26" t="n">
@@ -32663,7 +32663,7 @@
       </c>
       <c r="AX179" t="inlineStr">
         <is>
-          <t>3cr</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AY179" s="26" t="n">
@@ -32859,7 +32859,7 @@
       </c>
       <c r="AX180" s="18" t="inlineStr">
         <is>
-          <t>-6cr</t>
+          <t>-6</t>
         </is>
       </c>
       <c r="AY180" s="26" t="n">
@@ -33055,7 +33055,7 @@
       </c>
       <c r="AX181" s="18" t="inlineStr">
         <is>
-          <t>-59cr</t>
+          <t>-59</t>
         </is>
       </c>
       <c r="AY181" s="26" t="n">
@@ -33239,7 +33239,7 @@
       </c>
       <c r="AX182" t="inlineStr">
         <is>
-          <t>42cr</t>
+          <t>42</t>
         </is>
       </c>
       <c r="AY182" s="26" t="n">
@@ -33399,7 +33399,7 @@
       </c>
       <c r="AX183" s="18" t="inlineStr">
         <is>
-          <t>-79cr</t>
+          <t>-79</t>
         </is>
       </c>
       <c r="AY183" s="26" t="n">
@@ -33583,7 +33583,7 @@
       </c>
       <c r="AX184" t="inlineStr">
         <is>
-          <t>22cr</t>
+          <t>22</t>
         </is>
       </c>
       <c r="AY184" s="26" t="n">
@@ -33743,7 +33743,7 @@
       </c>
       <c r="AX185" s="18" t="inlineStr">
         <is>
-          <t>-6cr</t>
+          <t>-6</t>
         </is>
       </c>
       <c r="AY185" s="26" t="n">
@@ -33903,7 +33903,7 @@
       </c>
       <c r="AX186" s="18" t="inlineStr">
         <is>
-          <t>-53cr</t>
+          <t>-53</t>
         </is>
       </c>
       <c r="AY186" s="26" t="n">
@@ -34063,7 +34063,7 @@
       </c>
       <c r="AX187" s="18" t="inlineStr">
         <is>
-          <t>-181cr</t>
+          <t>-181</t>
         </is>
       </c>
       <c r="AY187" s="26" t="n">
@@ -34247,7 +34247,7 @@
       </c>
       <c r="AX188" s="18" t="inlineStr">
         <is>
-          <t>-20cr</t>
+          <t>-20</t>
         </is>
       </c>
       <c r="AY188" s="26" t="n">
@@ -34407,7 +34407,7 @@
       </c>
       <c r="AX189" s="18" t="inlineStr">
         <is>
-          <t>-117cr</t>
+          <t>-117</t>
         </is>
       </c>
       <c r="AY189" s="26" t="n">
@@ -34591,7 +34591,7 @@
       </c>
       <c r="AX190" s="18" t="inlineStr">
         <is>
-          <t>-2cr</t>
+          <t>-2</t>
         </is>
       </c>
       <c r="AY190" s="26" t="n">
@@ -34751,7 +34751,7 @@
       </c>
       <c r="AX191" s="18" t="inlineStr">
         <is>
-          <t>-66cr</t>
+          <t>-66</t>
         </is>
       </c>
       <c r="AY191" s="26" t="n">
@@ -34923,7 +34923,7 @@
       </c>
       <c r="AX192" s="18" t="inlineStr">
         <is>
-          <t>-12cr</t>
+          <t>-12</t>
         </is>
       </c>
       <c r="AY192" s="26" t="n">
@@ -35063,7 +35063,7 @@
       </c>
       <c r="AX193" s="18" t="inlineStr">
         <is>
-          <t>-120cr</t>
+          <t>-120</t>
         </is>
       </c>
       <c r="AY193" s="26" t="n">
@@ -35355,7 +35355,7 @@
       </c>
       <c r="AX195" s="18" t="inlineStr">
         <is>
-          <t>-18cr</t>
+          <t>-18</t>
         </is>
       </c>
       <c r="AY195" s="26" t="n">
@@ -35515,7 +35515,7 @@
       </c>
       <c r="AX196" s="18" t="inlineStr">
         <is>
-          <t>-9cr</t>
+          <t>-9</t>
         </is>
       </c>
       <c r="AY196" s="26" t="n">
@@ -35675,7 +35675,7 @@
       </c>
       <c r="AX197" s="18" t="inlineStr">
         <is>
-          <t>-64cr</t>
+          <t>-64</t>
         </is>
       </c>
       <c r="AY197" s="26" t="n">
@@ -35835,7 +35835,7 @@
       </c>
       <c r="AX198" s="18" t="inlineStr">
         <is>
-          <t>-1cr</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="AY198" s="26" t="n">
@@ -35995,7 +35995,7 @@
       </c>
       <c r="AX199" t="inlineStr">
         <is>
-          <t>33cr</t>
+          <t>33</t>
         </is>
       </c>
       <c r="AY199" s="26" t="n">
@@ -36135,7 +36135,7 @@
       </c>
       <c r="AX200" t="inlineStr">
         <is>
-          <t>34cr</t>
+          <t>34</t>
         </is>
       </c>
       <c r="AY200" s="26" t="n">
@@ -36295,7 +36295,7 @@
       </c>
       <c r="AX201" s="18" t="inlineStr">
         <is>
-          <t>-28cr</t>
+          <t>-28</t>
         </is>
       </c>
       <c r="AY201" s="26" t="n">
@@ -36455,7 +36455,7 @@
       </c>
       <c r="AX202" s="18" t="inlineStr">
         <is>
-          <t>-9cr</t>
+          <t>-9</t>
         </is>
       </c>
       <c r="AY202" s="26" t="n">
@@ -36651,7 +36651,7 @@
       </c>
       <c r="AX203" t="inlineStr">
         <is>
-          <t>16cr</t>
+          <t>16</t>
         </is>
       </c>
       <c r="AY203" s="26" t="n">
@@ -36847,7 +36847,7 @@
       </c>
       <c r="AX204" t="inlineStr">
         <is>
-          <t>9cr</t>
+          <t>9</t>
         </is>
       </c>
       <c r="AY204" s="26" t="n">
@@ -36987,7 +36987,7 @@
       </c>
       <c r="AX205" s="18" t="inlineStr">
         <is>
-          <t>-7cr</t>
+          <t>-7</t>
         </is>
       </c>
       <c r="AY205" s="26" t="n">
@@ -37159,7 +37159,7 @@
       </c>
       <c r="AX206" s="18" t="inlineStr">
         <is>
-          <t>-7cr</t>
+          <t>-7</t>
         </is>
       </c>
       <c r="AY206" s="26" t="n">
@@ -37299,7 +37299,7 @@
       </c>
       <c r="AX207" s="18" t="inlineStr">
         <is>
-          <t>-5cr</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="AY207" s="26" t="n">
@@ -37439,7 +37439,7 @@
       </c>
       <c r="AX208" s="18" t="inlineStr">
         <is>
-          <t>-22cr</t>
+          <t>-22</t>
         </is>
       </c>
       <c r="AY208" s="26" t="n">
@@ -37623,7 +37623,7 @@
       </c>
       <c r="AX209" s="18" t="inlineStr">
         <is>
-          <t>-13cr</t>
+          <t>-13</t>
         </is>
       </c>
       <c r="AY209" s="26" t="n">
@@ -37783,7 +37783,7 @@
       </c>
       <c r="AX210" s="18" t="inlineStr">
         <is>
-          <t>-41cr</t>
+          <t>-41</t>
         </is>
       </c>
       <c r="AY210" s="26" t="n">
@@ -37943,7 +37943,7 @@
       </c>
       <c r="AX211" s="18" t="inlineStr">
         <is>
-          <t>-65cr</t>
+          <t>-65</t>
         </is>
       </c>
       <c r="AY211" s="26" t="n">
@@ -38139,7 +38139,7 @@
       </c>
       <c r="AX212" s="18" t="inlineStr">
         <is>
-          <t>-15cr</t>
+          <t>-15</t>
         </is>
       </c>
       <c r="AY212" s="26" t="n">
@@ -38299,7 +38299,7 @@
       </c>
       <c r="AX213" s="18" t="inlineStr">
         <is>
-          <t>-44cr</t>
+          <t>-44</t>
         </is>
       </c>
       <c r="AY213" s="26" t="n">
@@ -38459,7 +38459,7 @@
       </c>
       <c r="AX214" s="18" t="inlineStr">
         <is>
-          <t>-40cr</t>
+          <t>-40</t>
         </is>
       </c>
       <c r="AY214" s="26" t="n">
@@ -38599,7 +38599,7 @@
       </c>
       <c r="AX215" t="inlineStr">
         <is>
-          <t>13cr</t>
+          <t>13</t>
         </is>
       </c>
       <c r="AY215" s="26" t="n">
@@ -38783,7 +38783,7 @@
       </c>
       <c r="AX216" s="18" t="inlineStr">
         <is>
-          <t>-9cr</t>
+          <t>-9</t>
         </is>
       </c>
       <c r="AY216" s="26" t="n">
@@ -38943,7 +38943,7 @@
       </c>
       <c r="AX217" t="inlineStr">
         <is>
-          <t>0cr</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY217" s="26" t="n">
@@ -39139,7 +39139,7 @@
       </c>
       <c r="AX218" t="inlineStr">
         <is>
-          <t>18cr</t>
+          <t>18</t>
         </is>
       </c>
       <c r="AY218" s="26" t="n">
@@ -39333,7 +39333,7 @@
       </c>
       <c r="AX219" s="18" t="inlineStr">
         <is>
-          <t>-6cr</t>
+          <t>-6</t>
         </is>
       </c>
       <c r="AY219" s="26" t="n">
@@ -39661,7 +39661,7 @@
       </c>
       <c r="AX221" t="inlineStr">
         <is>
-          <t>90cr</t>
+          <t>90</t>
         </is>
       </c>
       <c r="AY221" s="26" t="n">
@@ -39855,7 +39855,7 @@
       </c>
       <c r="AX222" t="inlineStr">
         <is>
-          <t>41cr</t>
+          <t>41</t>
         </is>
       </c>
       <c r="AY222" s="26" t="n">
@@ -40015,7 +40015,7 @@
       </c>
       <c r="AX223" t="inlineStr">
         <is>
-          <t>0cr</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY223" s="26" t="n">
@@ -40187,7 +40187,7 @@
       </c>
       <c r="AX224" s="18" t="inlineStr">
         <is>
-          <t>-108cr</t>
+          <t>-108</t>
         </is>
       </c>
       <c r="AY224" s="26" t="n">
@@ -40347,7 +40347,7 @@
       </c>
       <c r="AX225" s="18" t="inlineStr">
         <is>
-          <t>-59cr</t>
+          <t>-59</t>
         </is>
       </c>
       <c r="AY225" s="26" t="n">
@@ -40531,7 +40531,7 @@
       </c>
       <c r="AX226" s="18" t="inlineStr">
         <is>
-          <t>-2cr</t>
+          <t>-2</t>
         </is>
       </c>
       <c r="AY226" s="26" t="n">
@@ -40725,7 +40725,7 @@
       </c>
       <c r="AX227" s="18" t="inlineStr">
         <is>
-          <t>-48cr</t>
+          <t>-48</t>
         </is>
       </c>
       <c r="AY227" s="26" t="n">
@@ -40865,7 +40865,7 @@
       </c>
       <c r="AX228" s="18" t="inlineStr">
         <is>
-          <t>-64cr</t>
+          <t>-64</t>
         </is>
       </c>
       <c r="AY228" s="26" t="n">
@@ -41025,7 +41025,7 @@
       </c>
       <c r="AX229" s="18" t="inlineStr">
         <is>
-          <t>-332cr</t>
+          <t>-332</t>
         </is>
       </c>
       <c r="AY229" s="26" t="n">
@@ -41185,7 +41185,7 @@
       </c>
       <c r="AX230" s="18" t="inlineStr">
         <is>
-          <t>-5cr</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="AY230" s="26" t="n">
@@ -41345,7 +41345,7 @@
       </c>
       <c r="AX231" s="18" t="inlineStr">
         <is>
-          <t>-20cr</t>
+          <t>-20</t>
         </is>
       </c>
       <c r="AY231" s="26" t="n">
@@ -41505,7 +41505,7 @@
       </c>
       <c r="AX232" s="18" t="inlineStr">
         <is>
-          <t>-42cr</t>
+          <t>-42</t>
         </is>
       </c>
       <c r="AY232" s="26" t="n">
@@ -41665,7 +41665,7 @@
       </c>
       <c r="AX233" t="inlineStr">
         <is>
-          <t>23cr</t>
+          <t>23</t>
         </is>
       </c>
       <c r="AY233" s="26" t="n">
@@ -41825,7 +41825,7 @@
       </c>
       <c r="AX234" t="inlineStr">
         <is>
-          <t>16cr</t>
+          <t>16</t>
         </is>
       </c>
       <c r="AY234" s="26" t="n">
@@ -41985,7 +41985,7 @@
       </c>
       <c r="AX235" s="18" t="inlineStr">
         <is>
-          <t>-3cr</t>
+          <t>-3</t>
         </is>
       </c>
       <c r="AY235" s="26" t="n">
@@ -42181,7 +42181,7 @@
       </c>
       <c r="AX236" s="18" t="inlineStr">
         <is>
-          <t>-15cr</t>
+          <t>-15</t>
         </is>
       </c>
       <c r="AY236" s="26" t="n">
@@ -42341,7 +42341,7 @@
       </c>
       <c r="AX237" s="18" t="inlineStr">
         <is>
-          <t>-10cr</t>
+          <t>-10</t>
         </is>
       </c>
       <c r="AY237" s="26" t="n">
@@ -42481,7 +42481,7 @@
       </c>
       <c r="AX238" t="inlineStr">
         <is>
-          <t>24cr</t>
+          <t>24</t>
         </is>
       </c>
       <c r="AY238" s="26" t="n">
@@ -42641,7 +42641,7 @@
       </c>
       <c r="AX239" s="18" t="inlineStr">
         <is>
-          <t>-87cr</t>
+          <t>-87</t>
         </is>
       </c>
       <c r="AY239" s="26" t="n">
@@ -42837,7 +42837,7 @@
       </c>
       <c r="AX240" s="18" t="inlineStr">
         <is>
-          <t>-27cr</t>
+          <t>-27</t>
         </is>
       </c>
       <c r="AY240" s="26" t="n">
@@ -42977,7 +42977,7 @@
       </c>
       <c r="AX241" t="inlineStr">
         <is>
-          <t>64cr</t>
+          <t>64</t>
         </is>
       </c>
       <c r="AY241" s="26" t="n">
@@ -43161,7 +43161,7 @@
       </c>
       <c r="AX242" s="18" t="inlineStr">
         <is>
-          <t>-43cr</t>
+          <t>-43</t>
         </is>
       </c>
       <c r="AY242" s="26" t="n">
@@ -43333,7 +43333,7 @@
       </c>
       <c r="AX243" t="inlineStr">
         <is>
-          <t>307cr</t>
+          <t>307</t>
         </is>
       </c>
       <c r="AY243" s="26" t="n">
@@ -43517,7 +43517,7 @@
       </c>
       <c r="AX244" t="inlineStr">
         <is>
-          <t>265cr</t>
+          <t>265</t>
         </is>
       </c>
       <c r="AY244" s="26" t="n">
@@ -43657,7 +43657,7 @@
       </c>
       <c r="AX245" t="inlineStr">
         <is>
-          <t>7cr</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AY245" s="26" t="n">
@@ -43817,7 +43817,7 @@
       </c>
       <c r="AX246" s="18" t="inlineStr">
         <is>
-          <t>-38cr</t>
+          <t>-38</t>
         </is>
       </c>
       <c r="AY246" s="26" t="n">
@@ -44001,7 +44001,7 @@
       </c>
       <c r="AX247" s="18" t="inlineStr">
         <is>
-          <t>-20cr</t>
+          <t>-20</t>
         </is>
       </c>
       <c r="AY247" s="26" t="n">
@@ -44197,7 +44197,7 @@
       </c>
       <c r="AX248" s="18" t="inlineStr">
         <is>
-          <t>-106cr</t>
+          <t>-106</t>
         </is>
       </c>
       <c r="AY248" s="26" t="n">
@@ -44381,7 +44381,7 @@
       </c>
       <c r="AX249" t="inlineStr">
         <is>
-          <t>912cr</t>
+          <t>912</t>
         </is>
       </c>
       <c r="AY249" s="26" t="n">
@@ -44575,7 +44575,7 @@
       </c>
       <c r="AX250" t="inlineStr">
         <is>
-          <t>24cr</t>
+          <t>24</t>
         </is>
       </c>
       <c r="AY250" s="26" t="n">
@@ -44735,7 +44735,7 @@
       </c>
       <c r="AX251" t="inlineStr">
         <is>
-          <t>25cr</t>
+          <t>25</t>
         </is>
       </c>
       <c r="AY251" s="26" t="n">
@@ -44919,7 +44919,7 @@
       </c>
       <c r="AX252" s="18" t="inlineStr">
         <is>
-          <t>-78cr</t>
+          <t>-78</t>
         </is>
       </c>
       <c r="AY252" s="26" t="n">
@@ -45103,7 +45103,7 @@
       </c>
       <c r="AX253" t="inlineStr">
         <is>
-          <t>14cr</t>
+          <t>14</t>
         </is>
       </c>
       <c r="AY253" s="26" t="n">
@@ -45275,7 +45275,7 @@
       </c>
       <c r="AX254" s="18" t="inlineStr">
         <is>
-          <t>-19cr</t>
+          <t>-19</t>
         </is>
       </c>
       <c r="AY254" s="26" t="n">
@@ -45415,7 +45415,7 @@
       </c>
       <c r="AX255" s="18" t="inlineStr">
         <is>
-          <t>-17cr</t>
+          <t>-17</t>
         </is>
       </c>
       <c r="AY255" s="26" t="n">
@@ -45599,7 +45599,7 @@
       </c>
       <c r="AX256" t="inlineStr">
         <is>
-          <t>3cr</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AY256" s="26" t="n">
@@ -45739,7 +45739,7 @@
       </c>
       <c r="AX257" t="inlineStr">
         <is>
-          <t>62cr</t>
+          <t>62</t>
         </is>
       </c>
       <c r="AY257" s="26" t="n">
@@ -45933,7 +45933,7 @@
       </c>
       <c r="AX258" t="inlineStr">
         <is>
-          <t>350cr</t>
+          <t>350</t>
         </is>
       </c>
       <c r="AY258" s="26" t="n">
@@ -46073,7 +46073,7 @@
       </c>
       <c r="AX259" t="inlineStr">
         <is>
-          <t>29cr</t>
+          <t>29</t>
         </is>
       </c>
       <c r="AY259" s="26" t="n">
@@ -46213,7 +46213,7 @@
       </c>
       <c r="AX260" t="inlineStr">
         <is>
-          <t>12cr</t>
+          <t>12</t>
         </is>
       </c>
       <c r="AY260" s="26" t="n">
@@ -46385,7 +46385,7 @@
       </c>
       <c r="AX261" s="18" t="inlineStr">
         <is>
-          <t>-17cr</t>
+          <t>-17</t>
         </is>
       </c>
       <c r="AY261" s="26" t="n">
@@ -46581,7 +46581,7 @@
       </c>
       <c r="AX262" t="inlineStr">
         <is>
-          <t>9cr</t>
+          <t>9</t>
         </is>
       </c>
       <c r="AY262" s="26" t="n">
@@ -46775,7 +46775,7 @@
       </c>
       <c r="AX263" s="18" t="inlineStr">
         <is>
-          <t>-35cr</t>
+          <t>-35</t>
         </is>
       </c>
       <c r="AY263" s="26" t="n">
@@ -46935,7 +46935,7 @@
       </c>
       <c r="AX264" s="18" t="inlineStr">
         <is>
-          <t>-23cr</t>
+          <t>-23</t>
         </is>
       </c>
       <c r="AY264" s="26" t="n">
@@ -47131,7 +47131,7 @@
       </c>
       <c r="AX265" t="inlineStr">
         <is>
-          <t>3cr</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AY265" s="26" t="n">
@@ -47291,7 +47291,7 @@
       </c>
       <c r="AX266" s="18" t="inlineStr">
         <is>
-          <t>-10cr</t>
+          <t>-10</t>
         </is>
       </c>
       <c r="AY266" s="26" t="n">
@@ -47463,7 +47463,7 @@
       </c>
       <c r="AX267" t="inlineStr">
         <is>
-          <t>9cr</t>
+          <t>9</t>
         </is>
       </c>
       <c r="AY267" s="26" t="n">
@@ -47603,7 +47603,7 @@
       </c>
       <c r="AX268" t="inlineStr">
         <is>
-          <t>7cr</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AY268" s="26" t="n">
@@ -47743,7 +47743,7 @@
       </c>
       <c r="AX269" s="18" t="inlineStr">
         <is>
-          <t>-3cr</t>
+          <t>-3</t>
         </is>
       </c>
       <c r="AY269" s="26" t="n">
@@ -47915,7 +47915,7 @@
       </c>
       <c r="AX270" t="inlineStr">
         <is>
-          <t>50cr</t>
+          <t>50</t>
         </is>
       </c>
       <c r="AY270" s="26" t="n">
@@ -48075,7 +48075,7 @@
       </c>
       <c r="AX271" t="inlineStr">
         <is>
-          <t>24cr</t>
+          <t>24</t>
         </is>
       </c>
       <c r="AY271" s="26" t="n">
@@ -48215,7 +48215,7 @@
       </c>
       <c r="AX272" t="inlineStr">
         <is>
-          <t>28cr</t>
+          <t>28</t>
         </is>
       </c>
       <c r="AY272" s="26" t="n">
@@ -48399,7 +48399,7 @@
       </c>
       <c r="AX273" s="18" t="inlineStr">
         <is>
-          <t>-13cr</t>
+          <t>-13</t>
         </is>
       </c>
       <c r="AY273" s="26" t="n">
@@ -48559,7 +48559,7 @@
       </c>
       <c r="AX274" s="18" t="inlineStr">
         <is>
-          <t>-9cr</t>
+          <t>-9</t>
         </is>
       </c>
       <c r="AY274" s="26" t="n">
@@ -48755,7 +48755,7 @@
       </c>
       <c r="AX275" s="18" t="inlineStr">
         <is>
-          <t>-8cr</t>
+          <t>-8</t>
         </is>
       </c>
       <c r="AY275" s="26" t="n">
@@ -48927,7 +48927,7 @@
       </c>
       <c r="AX276" t="inlineStr">
         <is>
-          <t>32cr</t>
+          <t>32</t>
         </is>
       </c>
       <c r="AY276" s="26" t="n">
@@ -49087,7 +49087,7 @@
       </c>
       <c r="AX277" s="18" t="inlineStr">
         <is>
-          <t>-47cr</t>
+          <t>-47</t>
         </is>
       </c>
       <c r="AY277" s="26" t="n">
@@ -49247,7 +49247,7 @@
       </c>
       <c r="AX278" s="18" t="inlineStr">
         <is>
-          <t>-15cr</t>
+          <t>-15</t>
         </is>
       </c>
       <c r="AY278" s="26" t="n">
@@ -49539,7 +49539,7 @@
       </c>
       <c r="AX280" s="18" t="inlineStr">
         <is>
-          <t>-110cr</t>
+          <t>-110</t>
         </is>
       </c>
       <c r="AY280" s="26" t="n">
@@ -49699,7 +49699,7 @@
       </c>
       <c r="AX281" t="inlineStr">
         <is>
-          <t>30cr</t>
+          <t>30</t>
         </is>
       </c>
       <c r="AY281" s="26" t="n">
@@ -49859,7 +49859,7 @@
       </c>
       <c r="AX282" t="inlineStr">
         <is>
-          <t>27cr</t>
+          <t>27</t>
         </is>
       </c>
       <c r="AY282" s="26" t="n">
@@ -50175,7 +50175,7 @@
       </c>
       <c r="AX284" s="18" t="inlineStr">
         <is>
-          <t>-2cr</t>
+          <t>-2</t>
         </is>
       </c>
       <c r="AY284" s="26" t="n">
@@ -50371,7 +50371,7 @@
       </c>
       <c r="AX285" s="18" t="inlineStr">
         <is>
-          <t>-13cr</t>
+          <t>-13</t>
         </is>
       </c>
       <c r="AY285" s="26" t="n">
@@ -50531,7 +50531,7 @@
       </c>
       <c r="AX286" s="18" t="inlineStr">
         <is>
-          <t>-31cr</t>
+          <t>-31</t>
         </is>
       </c>
       <c r="AY286" s="26" t="n">
@@ -50691,7 +50691,7 @@
       </c>
       <c r="AX287" t="inlineStr">
         <is>
-          <t>13cr</t>
+          <t>13</t>
         </is>
       </c>
       <c r="AY287" s="26" t="n">
@@ -50875,7 +50875,7 @@
       </c>
       <c r="AX288" s="18" t="inlineStr">
         <is>
-          <t>-6cr</t>
+          <t>-6</t>
         </is>
       </c>
       <c r="AY288" s="26" t="n">
@@ -51035,7 +51035,7 @@
       </c>
       <c r="AX289" s="18" t="inlineStr">
         <is>
-          <t>-26cr</t>
+          <t>-26</t>
         </is>
       </c>
       <c r="AY289" s="26" t="n">
@@ -51219,7 +51219,7 @@
       </c>
       <c r="AX290" t="inlineStr">
         <is>
-          <t>3cr</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AY290" s="26" t="n">
@@ -51413,7 +51413,7 @@
       </c>
       <c r="AX291" s="18" t="inlineStr">
         <is>
-          <t>-61cr</t>
+          <t>-61</t>
         </is>
       </c>
       <c r="AY291" s="26" t="n">
@@ -51597,7 +51597,7 @@
       </c>
       <c r="AX292" s="18" t="inlineStr">
         <is>
-          <t>-34cr</t>
+          <t>-34</t>
         </is>
       </c>
       <c r="AY292" s="26" t="n">
@@ -51869,7 +51869,7 @@
       </c>
       <c r="AX294" t="inlineStr">
         <is>
-          <t>39cr</t>
+          <t>39</t>
         </is>
       </c>
       <c r="AY294" s="26" t="n">
@@ -52029,7 +52029,7 @@
       </c>
       <c r="AX295" s="18" t="inlineStr">
         <is>
-          <t>-120cr</t>
+          <t>-120</t>
         </is>
       </c>
       <c r="AY295" s="26" t="n">
@@ -52169,7 +52169,7 @@
       </c>
       <c r="AX296" t="inlineStr">
         <is>
-          <t>0cr</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY296" s="26" t="n">
@@ -52329,7 +52329,7 @@
       </c>
       <c r="AX297" s="18" t="inlineStr">
         <is>
-          <t>-14cr</t>
+          <t>-14</t>
         </is>
       </c>
       <c r="AY297" s="26" t="n">
@@ -52469,7 +52469,7 @@
       </c>
       <c r="AX298" t="inlineStr">
         <is>
-          <t>10cr</t>
+          <t>10</t>
         </is>
       </c>
       <c r="AY298" s="26" t="n">
@@ -52609,7 +52609,7 @@
       </c>
       <c r="AX299" s="18" t="inlineStr">
         <is>
-          <t>-13cr</t>
+          <t>-13</t>
         </is>
       </c>
       <c r="AY299" s="26" t="n">
@@ -52769,7 +52769,7 @@
       </c>
       <c r="AX300" s="18" t="inlineStr">
         <is>
-          <t>-30cr</t>
+          <t>-30</t>
         </is>
       </c>
       <c r="AY300" s="26" t="n">
@@ -52929,7 +52929,7 @@
       </c>
       <c r="AX301" t="inlineStr">
         <is>
-          <t>2cr</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AY301" s="26" t="n">
@@ -53069,7 +53069,7 @@
       </c>
       <c r="AX302" t="inlineStr">
         <is>
-          <t>8cr</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AY302" s="26" t="n">
@@ -53209,7 +53209,7 @@
       </c>
       <c r="AX303" t="inlineStr">
         <is>
-          <t>0cr</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY303" s="26" t="n">
@@ -53349,7 +53349,7 @@
       </c>
       <c r="AX304" t="inlineStr">
         <is>
-          <t>19cr</t>
+          <t>19</t>
         </is>
       </c>
       <c r="AY304" s="26" t="n">
@@ -53541,7 +53541,7 @@
       </c>
       <c r="AX305" t="inlineStr">
         <is>
-          <t>1cr</t>
+          <t>1</t>
         </is>
       </c>
       <c r="AY305" s="26" t="n">
@@ -53735,7 +53735,7 @@
       </c>
       <c r="AX306" s="18" t="inlineStr">
         <is>
-          <t>-31cr</t>
+          <t>-31</t>
         </is>
       </c>
       <c r="AY306" s="26" t="n">
@@ -53895,7 +53895,7 @@
       </c>
       <c r="AX307" s="18" t="inlineStr">
         <is>
-          <t>-33cr</t>
+          <t>-33</t>
         </is>
       </c>
       <c r="AY307" s="26" t="n">
@@ -54035,7 +54035,7 @@
       </c>
       <c r="AX308" t="inlineStr">
         <is>
-          <t>5cr</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AY308" s="26" t="n">
@@ -54229,7 +54229,7 @@
       </c>
       <c r="AX309" s="18" t="inlineStr">
         <is>
-          <t>-139cr</t>
+          <t>-139</t>
         </is>
       </c>
       <c r="AY309" s="26" t="n">
@@ -54425,7 +54425,7 @@
       </c>
       <c r="AX310" s="18" t="inlineStr">
         <is>
-          <t>-137cr</t>
+          <t>-137</t>
         </is>
       </c>
       <c r="AY310" s="26" t="n">
@@ -54621,7 +54621,7 @@
       </c>
       <c r="AX311" t="inlineStr">
         <is>
-          <t>1cr</t>
+          <t>1</t>
         </is>
       </c>
       <c r="AY311" s="26" t="n">
@@ -54949,7 +54949,7 @@
       </c>
       <c r="AX313" s="18" t="inlineStr">
         <is>
-          <t>-5cr</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="AY313" s="26" t="n">
@@ -55109,7 +55109,7 @@
       </c>
       <c r="AX314" t="inlineStr">
         <is>
-          <t>40cr</t>
+          <t>40</t>
         </is>
       </c>
       <c r="AY314" s="26" t="n">
@@ -55269,7 +55269,7 @@
       </c>
       <c r="AX315" t="inlineStr">
         <is>
-          <t>0cr</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY315" s="26" t="n">
@@ -55429,7 +55429,7 @@
       </c>
       <c r="AX316" s="18" t="inlineStr">
         <is>
-          <t>-8cr</t>
+          <t>-8</t>
         </is>
       </c>
       <c r="AY316" s="26" t="n">
@@ -55613,7 +55613,7 @@
       </c>
       <c r="AX317" s="18" t="inlineStr">
         <is>
-          <t>-4cr</t>
+          <t>-4</t>
         </is>
       </c>
       <c r="AY317" s="26" t="n">
@@ -55773,7 +55773,7 @@
       </c>
       <c r="AX318" s="18" t="inlineStr">
         <is>
-          <t>-17cr</t>
+          <t>-17</t>
         </is>
       </c>
       <c r="AY318" s="26" t="n">
@@ -55933,7 +55933,7 @@
       </c>
       <c r="AX319" s="18" t="inlineStr">
         <is>
-          <t>-33cr</t>
+          <t>-33</t>
         </is>
       </c>
       <c r="AY319" s="26" t="n">
@@ -56093,7 +56093,7 @@
       </c>
       <c r="AX320" s="18" t="inlineStr">
         <is>
-          <t>-44cr</t>
+          <t>-44</t>
         </is>
       </c>
       <c r="AY320" s="26" t="n">
@@ -56253,7 +56253,7 @@
       </c>
       <c r="AX321" s="18" t="inlineStr">
         <is>
-          <t>-33cr</t>
+          <t>-33</t>
         </is>
       </c>
       <c r="AY321" s="26" t="n">
@@ -56413,7 +56413,7 @@
       </c>
       <c r="AX322" s="18" t="inlineStr">
         <is>
-          <t>-21cr</t>
+          <t>-21</t>
         </is>
       </c>
       <c r="AY322" s="26" t="n">
@@ -56573,7 +56573,7 @@
       </c>
       <c r="AX323" t="inlineStr">
         <is>
-          <t>4cr</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AY323" s="26" t="n">
@@ -56733,7 +56733,7 @@
       </c>
       <c r="AX324" s="18" t="inlineStr">
         <is>
-          <t>-18cr</t>
+          <t>-18</t>
         </is>
       </c>
       <c r="AY324" s="26" t="n">
@@ -56893,7 +56893,7 @@
       </c>
       <c r="AX325" s="18" t="inlineStr">
         <is>
-          <t>-34cr</t>
+          <t>-34</t>
         </is>
       </c>
       <c r="AY325" s="26" t="n">
@@ -57077,7 +57077,7 @@
       </c>
       <c r="AX326" s="18" t="inlineStr">
         <is>
-          <t>-3cr</t>
+          <t>-3</t>
         </is>
       </c>
       <c r="AY326" s="26" t="n">
@@ -57271,7 +57271,7 @@
       </c>
       <c r="AX327" s="18" t="inlineStr">
         <is>
-          <t>-54cr</t>
+          <t>-54</t>
         </is>
       </c>
       <c r="AY327" s="26" t="n">
@@ -57431,7 +57431,7 @@
       </c>
       <c r="AX328" s="18" t="inlineStr">
         <is>
-          <t>-320cr</t>
+          <t>-320</t>
         </is>
       </c>
       <c r="AY328" s="26" t="n">
@@ -57627,7 +57627,7 @@
       </c>
       <c r="AX329" s="18" t="inlineStr">
         <is>
-          <t>-178cr</t>
+          <t>-178</t>
         </is>
       </c>
       <c r="AY329" s="26" t="n">
@@ -57787,7 +57787,7 @@
       </c>
       <c r="AX330" s="18" t="inlineStr">
         <is>
-          <t>-46cr</t>
+          <t>-46</t>
         </is>
       </c>
       <c r="AY330" s="26" t="n">
@@ -57947,7 +57947,7 @@
       </c>
       <c r="AX331" s="18" t="inlineStr">
         <is>
-          <t>-4cr</t>
+          <t>-4</t>
         </is>
       </c>
       <c r="AY331" s="26" t="n">
@@ -58107,7 +58107,7 @@
       </c>
       <c r="AX332" s="18" t="inlineStr">
         <is>
-          <t>-26cr</t>
+          <t>-26</t>
         </is>
       </c>
       <c r="AY332" s="26" t="n">
@@ -58303,7 +58303,7 @@
       </c>
       <c r="AX333" t="inlineStr">
         <is>
-          <t>5cr</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AY333" s="26" t="n">
@@ -58443,7 +58443,7 @@
       </c>
       <c r="AX334" t="inlineStr">
         <is>
-          <t>22cr</t>
+          <t>22</t>
         </is>
       </c>
       <c r="AY334" s="26" t="n">
@@ -58627,7 +58627,7 @@
       </c>
       <c r="AX335" t="inlineStr">
         <is>
-          <t>73cr</t>
+          <t>73</t>
         </is>
       </c>
       <c r="AY335" s="26" t="n">
@@ -58799,7 +58799,7 @@
       </c>
       <c r="AX336" s="18" t="inlineStr">
         <is>
-          <t>-41cr</t>
+          <t>-41</t>
         </is>
       </c>
       <c r="AY336" s="26" t="n">
@@ -58995,7 +58995,7 @@
       </c>
       <c r="AX337" t="inlineStr">
         <is>
-          <t>168cr</t>
+          <t>168</t>
         </is>
       </c>
       <c r="AY337" s="26" t="n">
@@ -59189,7 +59189,7 @@
       </c>
       <c r="AX338" t="inlineStr">
         <is>
-          <t>53cr</t>
+          <t>53</t>
         </is>
       </c>
       <c r="AY338" s="26" t="n">
@@ -59361,7 +59361,7 @@
       </c>
       <c r="AX339" s="18" t="inlineStr">
         <is>
-          <t>-11cr</t>
+          <t>-11</t>
         </is>
       </c>
       <c r="AY339" s="26" t="n">
@@ -59557,7 +59557,7 @@
       </c>
       <c r="AX340" s="18" t="inlineStr">
         <is>
-          <t>-35cr</t>
+          <t>-35</t>
         </is>
       </c>
       <c r="AY340" s="26" t="n">
@@ -59717,7 +59717,7 @@
       </c>
       <c r="AX341" s="18" t="inlineStr">
         <is>
-          <t>-90cr</t>
+          <t>-90</t>
         </is>
       </c>
       <c r="AY341" s="26" t="n">
@@ -59911,7 +59911,7 @@
       </c>
       <c r="AX342" s="18" t="inlineStr">
         <is>
-          <t>-41cr</t>
+          <t>-41</t>
         </is>
       </c>
       <c r="AY342" s="26" t="n">
@@ -60107,7 +60107,7 @@
       </c>
       <c r="AX343" t="inlineStr">
         <is>
-          <t>30cr</t>
+          <t>30</t>
         </is>
       </c>
       <c r="AY343" s="26" t="n">
@@ -60303,7 +60303,7 @@
       </c>
       <c r="AX344" t="inlineStr">
         <is>
-          <t>7cr</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AY344" s="26" t="n">
@@ -60499,7 +60499,7 @@
       </c>
       <c r="AX345" t="inlineStr">
         <is>
-          <t>0cr</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY345" s="26" t="n">
@@ -60659,7 +60659,7 @@
       </c>
       <c r="AX346" s="18" t="inlineStr">
         <is>
-          <t>-1cr</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="AY346" s="26" t="n">
@@ -60819,7 +60819,7 @@
       </c>
       <c r="AX347" s="18" t="inlineStr">
         <is>
-          <t>-15cr</t>
+          <t>-15</t>
         </is>
       </c>
       <c r="AY347" s="26" t="n">
@@ -60979,7 +60979,7 @@
       </c>
       <c r="AX348" s="18" t="inlineStr">
         <is>
-          <t>-8cr</t>
+          <t>-8</t>
         </is>
       </c>
       <c r="AY348" s="26" t="n">
@@ -61139,7 +61139,7 @@
       </c>
       <c r="AX349" t="inlineStr">
         <is>
-          <t>24cr</t>
+          <t>24</t>
         </is>
       </c>
       <c r="AY349" s="26" t="n">
@@ -61299,7 +61299,7 @@
       </c>
       <c r="AX350" t="inlineStr">
         <is>
-          <t>20cr</t>
+          <t>20</t>
         </is>
       </c>
       <c r="AY350" s="26" t="n">
@@ -61459,7 +61459,7 @@
       </c>
       <c r="AX351" s="18" t="inlineStr">
         <is>
-          <t>-2cr</t>
+          <t>-2</t>
         </is>
       </c>
       <c r="AY351" s="26" t="n">
@@ -61619,7 +61619,7 @@
       </c>
       <c r="AX352" t="inlineStr">
         <is>
-          <t>11cr</t>
+          <t>11</t>
         </is>
       </c>
       <c r="AZ352" s="26" t="n">
@@ -61753,7 +61753,7 @@
       </c>
       <c r="AX353" t="inlineStr">
         <is>
-          <t>6cr</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AY353" s="26" t="n">
@@ -62035,7 +62035,7 @@
       </c>
       <c r="AX355" s="18" t="inlineStr">
         <is>
-          <t>-227cr</t>
+          <t>-227</t>
         </is>
       </c>
       <c r="AY355" s="26" t="n">
@@ -62175,7 +62175,7 @@
       </c>
       <c r="AX356" t="inlineStr">
         <is>
-          <t>55cr</t>
+          <t>55</t>
         </is>
       </c>
       <c r="AY356" s="26" t="n">
@@ -62359,7 +62359,7 @@
       </c>
       <c r="AX357" s="18" t="inlineStr">
         <is>
-          <t>-44cr</t>
+          <t>-44</t>
         </is>
       </c>
       <c r="AY357" s="26" t="n">
@@ -62519,7 +62519,7 @@
       </c>
       <c r="AX358" s="18" t="inlineStr">
         <is>
-          <t>-24cr</t>
+          <t>-24</t>
         </is>
       </c>
       <c r="AY358" s="26" t="n">
@@ -62703,7 +62703,7 @@
       </c>
       <c r="AX359" t="inlineStr">
         <is>
-          <t>5cr</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AY359" s="26" t="n">
@@ -62887,7 +62887,7 @@
       </c>
       <c r="AX360" t="inlineStr">
         <is>
-          <t>118cr</t>
+          <t>118</t>
         </is>
       </c>
       <c r="AY360" s="26" t="n">
@@ -63083,7 +63083,7 @@
       </c>
       <c r="AX361" s="18" t="inlineStr">
         <is>
-          <t>-305cr</t>
+          <t>-305</t>
         </is>
       </c>
       <c r="AY361" s="26" t="n">
@@ -63277,7 +63277,7 @@
       </c>
       <c r="AX362" s="18" t="inlineStr">
         <is>
-          <t>-187cr</t>
+          <t>-187</t>
         </is>
       </c>
       <c r="AY362" s="26" t="n">
@@ -63605,7 +63605,7 @@
       </c>
       <c r="AX364" s="18" t="inlineStr">
         <is>
-          <t>-275cr</t>
+          <t>-275</t>
         </is>
       </c>
       <c r="AY364" s="26" t="n">
@@ -63801,7 +63801,7 @@
       </c>
       <c r="AX365" s="18" t="inlineStr">
         <is>
-          <t>-34cr</t>
+          <t>-34</t>
         </is>
       </c>
       <c r="AY365" s="26" t="n">
@@ -63985,7 +63985,7 @@
       </c>
       <c r="AX366" t="inlineStr">
         <is>
-          <t>263cr</t>
+          <t>263</t>
         </is>
       </c>
       <c r="AY366" s="26" t="n">
@@ -64169,7 +64169,7 @@
       </c>
       <c r="AX367" s="18" t="inlineStr">
         <is>
-          <t>-38cr</t>
+          <t>-38</t>
         </is>
       </c>
       <c r="AY367" s="26" t="n">
@@ -64329,7 +64329,7 @@
       </c>
       <c r="AX368" s="18" t="inlineStr">
         <is>
-          <t>-42cr</t>
+          <t>-42</t>
         </is>
       </c>
       <c r="AY368" s="26" t="n">
@@ -64523,7 +64523,7 @@
       </c>
       <c r="AX369" s="18" t="inlineStr">
         <is>
-          <t>-180cr</t>
+          <t>-180</t>
         </is>
       </c>
       <c r="AY369" s="26" t="n">
@@ -64707,7 +64707,7 @@
       </c>
       <c r="AX370" t="inlineStr">
         <is>
-          <t>2cr</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AY370" s="26" t="n">
@@ -64879,7 +64879,7 @@
       </c>
       <c r="AX371" s="18" t="inlineStr">
         <is>
-          <t>-14cr</t>
+          <t>-14</t>
         </is>
       </c>
       <c r="AY371" s="26" t="n">
@@ -65019,7 +65019,7 @@
       </c>
       <c r="AX372" t="inlineStr">
         <is>
-          <t>169cr</t>
+          <t>169</t>
         </is>
       </c>
       <c r="AY372" s="26" t="n">
@@ -65179,7 +65179,7 @@
       </c>
       <c r="AX373" s="18" t="inlineStr">
         <is>
-          <t>-42cr</t>
+          <t>-42</t>
         </is>
       </c>
       <c r="AY373" s="26" t="n">
@@ -65375,7 +65375,7 @@
       </c>
       <c r="AX374" s="18" t="inlineStr">
         <is>
-          <t>-323cr</t>
+          <t>-323</t>
         </is>
       </c>
       <c r="AY374" s="26" t="n">
@@ -65547,7 +65547,7 @@
       </c>
       <c r="AX375" s="18" t="inlineStr">
         <is>
-          <t>-40cr</t>
+          <t>-40</t>
         </is>
       </c>
       <c r="AY375" s="26" t="n">
@@ -65707,7 +65707,7 @@
       </c>
       <c r="AX376" t="inlineStr">
         <is>
-          <t>6cr</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AY376" s="26" t="n">
@@ -65901,7 +65901,7 @@
       </c>
       <c r="AX377" s="18" t="inlineStr">
         <is>
-          <t>-44cr</t>
+          <t>-44</t>
         </is>
       </c>
       <c r="AY377" s="26" t="n">
@@ -66085,7 +66085,7 @@
       </c>
       <c r="AX378" s="18" t="inlineStr">
         <is>
-          <t>-65cr</t>
+          <t>-65</t>
         </is>
       </c>
       <c r="AY378" s="26" t="n">
@@ -66281,7 +66281,7 @@
       </c>
       <c r="AX379" s="18" t="inlineStr">
         <is>
-          <t>-27cr</t>
+          <t>-27</t>
         </is>
       </c>
       <c r="AY379" s="26" t="n">
@@ -66563,7 +66563,7 @@
       </c>
       <c r="AX381" t="inlineStr">
         <is>
-          <t>61cr</t>
+          <t>61</t>
         </is>
       </c>
       <c r="AY381" s="26" t="n">
@@ -66735,7 +66735,7 @@
       </c>
       <c r="AX382" t="inlineStr">
         <is>
-          <t>174cr</t>
+          <t>174</t>
         </is>
       </c>
       <c r="AY382" s="26" t="n">
@@ -66931,7 +66931,7 @@
       </c>
       <c r="AX383" t="inlineStr">
         <is>
-          <t>22cr</t>
+          <t>22</t>
         </is>
       </c>
       <c r="AY383" s="26" t="n">
@@ -67091,7 +67091,7 @@
       </c>
       <c r="AX384" s="18" t="inlineStr">
         <is>
-          <t>-20cr</t>
+          <t>-20</t>
         </is>
       </c>
       <c r="AY384" s="26" t="n">
@@ -67263,7 +67263,7 @@
       </c>
       <c r="AX385" t="inlineStr">
         <is>
-          <t>1cr</t>
+          <t>1</t>
         </is>
       </c>
       <c r="AY385" s="26" t="n">
@@ -67459,7 +67459,7 @@
       </c>
       <c r="AX386" t="inlineStr">
         <is>
-          <t>1cr</t>
+          <t>1</t>
         </is>
       </c>
       <c r="AY386" s="26" t="n">
@@ -67653,7 +67653,7 @@
       </c>
       <c r="AX387" s="18" t="inlineStr">
         <is>
-          <t>-5cr</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="AY387" s="26" t="n">
@@ -67849,7 +67849,7 @@
       </c>
       <c r="AX388" t="inlineStr">
         <is>
-          <t>225cr</t>
+          <t>225</t>
         </is>
       </c>
       <c r="AY388" s="26" t="n">
@@ -68021,7 +68021,7 @@
       </c>
       <c r="AX389" t="inlineStr">
         <is>
-          <t>3cr</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AY389" s="26" t="n">
@@ -68215,7 +68215,7 @@
       </c>
       <c r="AX390" s="18" t="inlineStr">
         <is>
-          <t>-31cr</t>
+          <t>-31</t>
         </is>
       </c>
       <c r="AY390" s="26" t="n">
@@ -68399,7 +68399,7 @@
       </c>
       <c r="AX391" s="18" t="inlineStr">
         <is>
-          <t>-5cr</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="AY391" s="26" t="n">
@@ -68539,7 +68539,7 @@
       </c>
       <c r="AX392" t="inlineStr">
         <is>
-          <t>43cr</t>
+          <t>43</t>
         </is>
       </c>
       <c r="AY392" s="26" t="n">
@@ -68735,7 +68735,7 @@
       </c>
       <c r="AX393" s="18" t="inlineStr">
         <is>
-          <t>-35cr</t>
+          <t>-35</t>
         </is>
       </c>
       <c r="AY393" s="26" t="n">
@@ -68931,7 +68931,7 @@
       </c>
       <c r="AX394" s="18" t="inlineStr">
         <is>
-          <t>-5cr</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="AY394" s="26" t="n">
@@ -69127,7 +69127,7 @@
       </c>
       <c r="AX395" s="18" t="inlineStr">
         <is>
-          <t>7cr</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AY395" s="26" t="n">
@@ -69323,7 +69323,7 @@
       </c>
       <c r="AX396" t="inlineStr">
         <is>
-          <t>9cr</t>
+          <t>9</t>
         </is>
       </c>
       <c r="AY396" s="26" t="n">
@@ -69507,7 +69507,7 @@
       </c>
       <c r="AX397" t="inlineStr">
         <is>
-          <t>3cr</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AY397" s="26" t="n">

</xml_diff>